<commit_message>
feature: adiciona renomeador de arquivos feito em python.
</commit_message>
<xml_diff>
--- a/01_Excel_PowerQuery/Excel Impressionador - Hashtag/planilhas/funcao_COUNTIFS.xlsx
+++ b/01_Excel_PowerQuery/Excel Impressionador - Hashtag/planilhas/funcao_COUNTIFS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joaof\Desktop\Excel Impressionador 2021\Módulo 8 - Funções Mercado de Trabalho\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E79C64-1286-485D-968C-EE0DC01F6608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F908A640-9FF3-46D6-8ECD-F4D226521430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{3D2557DA-CD0B-48AD-8EFD-8912689B8782}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{3D2557DA-CD0B-48AD-8EFD-8912689B8782}"/>
   </bookViews>
   <sheets>
     <sheet name="CONT.SES" sheetId="2" r:id="rId1"/>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pratica!$A$1:$E$50</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -31,6 +31,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -38,201 +40,102 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="95">
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t>Equipe</t>
+  </si>
+  <si>
+    <t>Sexo</t>
+  </si>
+  <si>
+    <t>Faturamento</t>
+  </si>
+  <si>
+    <t>Cor</t>
+  </si>
+  <si>
+    <t>Preta</t>
+  </si>
+  <si>
+    <t>Pedro Martins</t>
+  </si>
+  <si>
+    <t>Azul</t>
+  </si>
+  <si>
+    <t>Masculino</t>
+  </si>
+  <si>
+    <t>Quantidade</t>
+  </si>
+  <si>
+    <t>Camila Cury</t>
+  </si>
+  <si>
+    <t>Amarela</t>
+  </si>
+  <si>
+    <t>Feminino</t>
+  </si>
+  <si>
+    <t>Luiza França</t>
+  </si>
+  <si>
+    <t>Amanda Egler</t>
+  </si>
+  <si>
+    <t>Sergio Tranjan</t>
+  </si>
+  <si>
+    <t>Felipe Almeida</t>
+  </si>
+  <si>
+    <t>Caio Junqueira</t>
+  </si>
+  <si>
+    <t>Lais Azevedo</t>
+  </si>
+  <si>
+    <t>Tainá Motta</t>
+  </si>
+  <si>
+    <t>Jurandir Piscatella</t>
+  </si>
+  <si>
+    <t>Wilson Arrascaeta</t>
+  </si>
+  <si>
+    <t>Tomás Melo</t>
+  </si>
+  <si>
+    <t>Mariana Ferreira</t>
+  </si>
   <si>
     <t>Registro</t>
   </si>
   <si>
-    <t>Analista Pleno</t>
-  </si>
-  <si>
-    <t>Analista Pro</t>
+    <t>Cargo</t>
+  </si>
+  <si>
+    <t>Área</t>
+  </si>
+  <si>
+    <t>Salário</t>
+  </si>
+  <si>
+    <t>Contratação</t>
+  </si>
+  <si>
+    <t>PF15337</t>
   </si>
   <si>
     <t>Coordenador</t>
   </si>
   <si>
-    <t>Gerente</t>
-  </si>
-  <si>
-    <t>Estagiário</t>
-  </si>
-  <si>
-    <t>FS14645</t>
-  </si>
-  <si>
-    <t>YY71148</t>
-  </si>
-  <si>
-    <t>JY48754</t>
-  </si>
-  <si>
-    <t>JY92653</t>
-  </si>
-  <si>
-    <t>PP76167</t>
-  </si>
-  <si>
-    <t>YJ83493</t>
-  </si>
-  <si>
-    <t>YY62461</t>
-  </si>
-  <si>
-    <t>YF59381</t>
-  </si>
-  <si>
-    <t>PS11194</t>
-  </si>
-  <si>
-    <t>YJ95237</t>
-  </si>
-  <si>
-    <t>FS39573</t>
-  </si>
-  <si>
-    <t>FY58574</t>
-  </si>
-  <si>
-    <t>PY34116</t>
-  </si>
-  <si>
-    <t>YY35665</t>
-  </si>
-  <si>
-    <t>PF15337</t>
-  </si>
-  <si>
-    <t>SS14724</t>
-  </si>
-  <si>
-    <t>FS17182</t>
-  </si>
-  <si>
-    <t>PF14125</t>
-  </si>
-  <si>
-    <t>YY49857</t>
-  </si>
-  <si>
-    <t>FY41531</t>
-  </si>
-  <si>
-    <t>SJ71953</t>
-  </si>
-  <si>
-    <t>JP31187</t>
-  </si>
-  <si>
-    <t>YF65454</t>
-  </si>
-  <si>
-    <t>JF14563</t>
-  </si>
-  <si>
-    <t>PJ12117</t>
-  </si>
-  <si>
-    <t>PY13951</t>
-  </si>
-  <si>
-    <t>FS17453</t>
-  </si>
-  <si>
-    <t>SS26785</t>
-  </si>
-  <si>
-    <t>JP91247</t>
-  </si>
-  <si>
-    <t>YP58227</t>
-  </si>
-  <si>
-    <t>YY47449</t>
-  </si>
-  <si>
-    <t>YS42793</t>
-  </si>
-  <si>
-    <t>FY11681</t>
-  </si>
-  <si>
-    <t>YJ68539</t>
-  </si>
-  <si>
-    <t>YF91336</t>
-  </si>
-  <si>
-    <t>FP15212</t>
-  </si>
-  <si>
-    <t>PF82962</t>
-  </si>
-  <si>
-    <t>YF53139</t>
-  </si>
-  <si>
-    <t>YP41282</t>
-  </si>
-  <si>
-    <t>SY65154</t>
-  </si>
-  <si>
-    <t>YP61865</t>
-  </si>
-  <si>
-    <t>YY82624</t>
-  </si>
-  <si>
-    <t>JS27876</t>
-  </si>
-  <si>
-    <t>YF48464</t>
-  </si>
-  <si>
-    <t>PY64522</t>
-  </si>
-  <si>
-    <t>FS82397</t>
-  </si>
-  <si>
-    <t>PY15333</t>
-  </si>
-  <si>
-    <t>PY93318</t>
-  </si>
-  <si>
-    <t>PP53616</t>
-  </si>
-  <si>
-    <t>Salário</t>
-  </si>
-  <si>
-    <t>Cargo</t>
-  </si>
-  <si>
-    <t>Financeiro</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>Comercial</t>
-  </si>
-  <si>
-    <t>Administrativo</t>
-  </si>
-  <si>
     <t>Suporte</t>
-  </si>
-  <si>
-    <t>Gestão de Pessoas</t>
-  </si>
-  <si>
-    <t>Contratação</t>
-  </si>
-  <si>
-    <t>Área</t>
   </si>
   <si>
     <r>
@@ -261,6 +164,33 @@
     </r>
   </si>
   <si>
+    <t>PY13951</t>
+  </si>
+  <si>
+    <t>Estagiário</t>
+  </si>
+  <si>
+    <t>Financeiro</t>
+  </si>
+  <si>
+    <t>PP76167</t>
+  </si>
+  <si>
+    <t>Analista Pro</t>
+  </si>
+  <si>
+    <t>YF91336</t>
+  </si>
+  <si>
+    <t>Gerente</t>
+  </si>
+  <si>
+    <t>Gestão de Pessoas</t>
+  </si>
+  <si>
+    <t>FS14645</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Quantas pessoas foram contratadas após </t>
     </r>
@@ -285,6 +215,27 @@
       </rPr>
       <t>?</t>
     </r>
+  </si>
+  <si>
+    <t>JP91247</t>
+  </si>
+  <si>
+    <t>Comercial</t>
+  </si>
+  <si>
+    <t>PJ12117</t>
+  </si>
+  <si>
+    <t>PP53616</t>
+  </si>
+  <si>
+    <t>Analista Pleno</t>
+  </si>
+  <si>
+    <t>YF48464</t>
+  </si>
+  <si>
+    <t>Administrativo</t>
   </si>
   <si>
     <r>
@@ -334,6 +285,36 @@
     </r>
   </si>
   <si>
+    <t>YS42793</t>
+  </si>
+  <si>
+    <t>YY62461</t>
+  </si>
+  <si>
+    <t>JY92653</t>
+  </si>
+  <si>
+    <t>JY48754</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Quantos analistas a empresa possui?</t>
+  </si>
+  <si>
+    <t>YJ68539</t>
+  </si>
+  <si>
+    <t>JS27876</t>
+  </si>
+  <si>
+    <t>YJ83493</t>
+  </si>
+  <si>
+    <t>YY82624</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Quantas pessoas do </t>
     </r>
@@ -360,73 +341,103 @@
     </r>
   </si>
   <si>
-    <t>Quantos analistas a empresa possui?</t>
-  </si>
-  <si>
-    <t>Nome</t>
-  </si>
-  <si>
-    <t>Equipe</t>
-  </si>
-  <si>
-    <t>Sexo</t>
-  </si>
-  <si>
-    <t>Faturamento</t>
-  </si>
-  <si>
-    <t>Pedro Martins</t>
-  </si>
-  <si>
-    <t>Camila Cury</t>
-  </si>
-  <si>
-    <t>Luiza França</t>
-  </si>
-  <si>
-    <t>Amanda Egler</t>
-  </si>
-  <si>
-    <t>Sergio Tranjan</t>
-  </si>
-  <si>
-    <t>Felipe Almeida</t>
-  </si>
-  <si>
-    <t>Caio Junqueira</t>
-  </si>
-  <si>
-    <t>Lais Azevedo</t>
-  </si>
-  <si>
-    <t>Tainá Motta</t>
-  </si>
-  <si>
-    <t>Jurandir Piscatella</t>
-  </si>
-  <si>
-    <t>Wilson Arrascaeta</t>
-  </si>
-  <si>
-    <t>Tomás Melo</t>
-  </si>
-  <si>
-    <t>Azul</t>
-  </si>
-  <si>
-    <t>Amarela</t>
-  </si>
-  <si>
-    <t>Preta</t>
-  </si>
-  <si>
-    <t>Masculino</t>
-  </si>
-  <si>
-    <t>Feminino</t>
-  </si>
-  <si>
-    <t>Mariana Ferreira</t>
+    <t>YP41282</t>
+  </si>
+  <si>
+    <t>YY35665</t>
+  </si>
+  <si>
+    <t>Setor:</t>
+  </si>
+  <si>
+    <t>YP58227</t>
+  </si>
+  <si>
+    <t>PF82962</t>
+  </si>
+  <si>
+    <t>SJ71953</t>
+  </si>
+  <si>
+    <t>YF53139</t>
+  </si>
+  <si>
+    <t>PS11194</t>
+  </si>
+  <si>
+    <t>JP31187</t>
+  </si>
+  <si>
+    <t>FS17453</t>
+  </si>
+  <si>
+    <t>YY49857</t>
+  </si>
+  <si>
+    <t>PY34116</t>
+  </si>
+  <si>
+    <t>PY15333</t>
+  </si>
+  <si>
+    <t>JF14563</t>
+  </si>
+  <si>
+    <t>YY71148</t>
+  </si>
+  <si>
+    <t>FY58574</t>
+  </si>
+  <si>
+    <t>PY93318</t>
+  </si>
+  <si>
+    <t>YY47449</t>
+  </si>
+  <si>
+    <t>FS82397</t>
+  </si>
+  <si>
+    <t>PY64522</t>
+  </si>
+  <si>
+    <t>YF65454</t>
+  </si>
+  <si>
+    <t>FS17182</t>
+  </si>
+  <si>
+    <t>SY65154</t>
+  </si>
+  <si>
+    <t>FY11681</t>
+  </si>
+  <si>
+    <t>FS39573</t>
+  </si>
+  <si>
+    <t>FP15212</t>
+  </si>
+  <si>
+    <t>SS26785</t>
+  </si>
+  <si>
+    <t>YF59381</t>
+  </si>
+  <si>
+    <t>YP61865</t>
+  </si>
+  <si>
+    <t>PF14125</t>
+  </si>
+  <si>
+    <t>FY41531</t>
+  </si>
+  <si>
+    <t>SS14724</t>
+  </si>
+  <si>
+    <t>YJ95237</t>
   </si>
 </sst>
 </file>
@@ -436,7 +447,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -515,7 +526,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -531,9 +542,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -569,7 +577,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -865,207 +873,234 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37263547-D7E7-4AC6-B262-BC90CCAE7898}">
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="19.77734375" customWidth="1"/>
-    <col min="2" max="4" width="15.77734375" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="4" width="15.7109375" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D2" s="14">
+        <v>8</v>
+      </c>
+      <c r="D2" s="13">
         <v>11555</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <f>COUNTIFS(B2:B14,G1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D3" s="14">
+        <v>12</v>
+      </c>
+      <c r="D3" s="13">
         <v>23113</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D4" s="14">
+        <v>12</v>
+      </c>
+      <c r="D4" s="13">
         <v>2585</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>86</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D5" s="14">
+        <v>12</v>
+      </c>
+      <c r="D5" s="13">
         <v>32635</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5">
+        <f>COUNTIFS(B2:B14,G1,C2:C14,"Feminino")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>89</v>
-      </c>
-      <c r="D6" s="14">
+        <v>8</v>
+      </c>
+      <c r="D6" s="13">
         <v>22529</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
+        <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>89</v>
-      </c>
-      <c r="D7" s="14">
+        <v>8</v>
+      </c>
+      <c r="D7" s="13">
         <v>33740</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>80</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>86</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
-      </c>
-      <c r="D8" s="14">
+        <v>8</v>
+      </c>
+      <c r="D8" s="13">
         <v>44566</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>81</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>90</v>
-      </c>
-      <c r="D9" s="14">
+        <v>12</v>
+      </c>
+      <c r="D9" s="13">
         <v>16756</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>88</v>
+        <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>90</v>
-      </c>
-      <c r="D10" s="14">
+        <v>12</v>
+      </c>
+      <c r="D10" s="13">
         <v>24899</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>89</v>
-      </c>
-      <c r="D11" s="14">
+        <v>8</v>
+      </c>
+      <c r="D11" s="13">
         <v>25086</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
-      </c>
-      <c r="D12" s="14">
+        <v>8</v>
+      </c>
+      <c r="D12" s="13">
         <v>6318</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>86</v>
+        <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>89</v>
-      </c>
-      <c r="D13" s="14">
+        <v>8</v>
+      </c>
+      <c r="D13" s="13">
         <v>15710</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>88</v>
+        <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
-      </c>
-      <c r="D14" s="14">
+        <v>12</v>
+      </c>
+      <c r="D14" s="13">
         <v>23626</v>
       </c>
     </row>
@@ -1077,46 +1112,46 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29FEF772-DFD0-4036-8B65-DBF82BF00CE4}">
   <dimension ref="A1:K50"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="2" customWidth="1"/>
     <col min="2" max="2" width="17" style="2" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="5" width="13.5546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="2.5546875" customWidth="1"/>
+    <col min="4" max="5" width="13.5703125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="2.5703125" customWidth="1"/>
     <col min="7" max="7" width="4" customWidth="1"/>
-    <col min="8" max="8" width="18.21875" customWidth="1"/>
+    <col min="8" max="8" width="18.28515625" customWidth="1"/>
     <col min="9" max="9" width="9" customWidth="1"/>
-    <col min="10" max="11" width="18.21875" customWidth="1"/>
-    <col min="12" max="12" width="16.77734375" customWidth="1"/>
+    <col min="10" max="11" width="18.28515625" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11">
+      <c r="A1" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" s="3" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="D2" s="4">
         <v>12500</v>
@@ -1124,25 +1159,25 @@
       <c r="E2" s="5">
         <v>42769</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="8">
         <v>1</v>
       </c>
-      <c r="H2" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H2" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+    </row>
+    <row r="3" spans="1:11" ht="15">
       <c r="A3" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D3" s="4">
         <v>1200</v>
@@ -1151,15 +1186,15 @@
         <v>42777</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="15">
       <c r="A4" s="3" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="D4" s="4">
         <v>4600</v>
@@ -1167,17 +1202,20 @@
       <c r="E4" s="5">
         <v>42811</v>
       </c>
-      <c r="H4" s="7"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H4">
+        <f>COUNTIFS(B:B,"Coordenador")</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="D5" s="4">
         <v>16000</v>
@@ -1187,15 +1225,15 @@
       </c>
       <c r="G5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="D6" s="4">
         <v>12500</v>
@@ -1203,25 +1241,25 @@
       <c r="E6" s="5">
         <v>42837</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="8">
         <v>2</v>
       </c>
-      <c r="H6" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H6" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+    </row>
+    <row r="7" spans="1:11" ht="15">
       <c r="A7" s="3" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="D7" s="4">
         <v>16000</v>
@@ -1230,15 +1268,15 @@
         <v>42904</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15">
       <c r="A8" s="3" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D8" s="4">
         <v>4600</v>
@@ -1246,17 +1284,20 @@
       <c r="E8" s="5">
         <v>42925</v>
       </c>
-      <c r="H8" s="7"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H8">
+        <f>COUNTIFS(E:E,"&gt;31/12/2018")</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" s="3" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D9" s="4">
         <v>3200</v>
@@ -1265,15 +1306,15 @@
         <v>42932</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11">
       <c r="A10" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>49</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="D10" s="4">
         <v>3200</v>
@@ -1281,25 +1322,25 @@
       <c r="E10" s="5">
         <v>43049</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="8">
         <v>3</v>
       </c>
-      <c r="H10" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H10" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+    </row>
+    <row r="11" spans="1:11" ht="15">
       <c r="A11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>2</v>
-      </c>
       <c r="C11" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D11" s="4">
         <v>4600</v>
@@ -1308,15 +1349,15 @@
         <v>43112</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="15">
       <c r="A12" s="3" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="D12" s="4">
         <v>3200</v>
@@ -1324,17 +1365,20 @@
       <c r="E12" s="5">
         <v>43143</v>
       </c>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H12">
+        <f>COUNTIFS(C:C,"Marketing",D:D,"&gt;4000")</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" s="3" t="s">
-        <v>9</v>
+        <v>53</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="D13" s="4">
         <v>1200</v>
@@ -1343,15 +1387,15 @@
         <v>43146</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11">
       <c r="A14" s="3" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D14" s="4">
         <v>12500</v>
@@ -1359,25 +1403,25 @@
       <c r="E14" s="5">
         <v>43153</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="8">
         <v>4</v>
       </c>
-      <c r="H14" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H14" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+    </row>
+    <row r="15" spans="1:11" ht="15">
       <c r="A15" s="3" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D15" s="4">
         <v>1200</v>
@@ -1386,15 +1430,15 @@
         <v>43168</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="15">
       <c r="A16" s="3" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D16" s="4">
         <v>1200</v>
@@ -1402,17 +1446,20 @@
       <c r="E16" s="5">
         <v>43215</v>
       </c>
-      <c r="H16" s="7"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H16">
+        <f>COUNTIFS(B:B,"*Analista*")</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
       <c r="A17" s="3" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D17" s="4">
         <v>12500</v>
@@ -1421,15 +1468,15 @@
         <v>43228</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11">
       <c r="A18" s="3" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="D18" s="4">
         <v>1200</v>
@@ -1437,25 +1484,25 @@
       <c r="E18" s="5">
         <v>43236</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="8">
         <v>5</v>
       </c>
-      <c r="H18" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H18" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+    </row>
+    <row r="19" spans="1:11">
       <c r="A19" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="D19" s="4">
         <v>12500</v>
@@ -1464,15 +1511,15 @@
         <v>43272</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11">
       <c r="A20" s="3" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="D20" s="4">
         <v>3200</v>
@@ -1480,20 +1527,29 @@
       <c r="E20" s="5">
         <v>43317</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="H20" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="I20" s="10">
+        <f>COUNTIFS(C:C,$K$20,B:B,H20)</f>
         <v>3</v>
       </c>
-      <c r="I20" s="11"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J20" t="s">
+        <v>64</v>
+      </c>
+      <c r="K20" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
       <c r="A21" s="3" t="s">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="D21" s="4">
         <v>1200</v>
@@ -1501,20 +1557,23 @@
       <c r="E21" s="5">
         <v>43328</v>
       </c>
-      <c r="H21" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="I21" s="11"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H21" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="I21" s="10">
+        <f t="shared" ref="I21:I24" si="0">COUNTIFS(C:C,$K$20,B:B,H21)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
       <c r="A22" s="3" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D22" s="4">
         <v>4600</v>
@@ -1522,20 +1581,23 @@
       <c r="E22" s="5">
         <v>43413</v>
       </c>
-      <c r="H22" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="I22" s="11"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H22" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="I22" s="10">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
       <c r="A23" s="3" t="s">
-        <v>26</v>
+        <v>67</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D23" s="4">
         <v>4600</v>
@@ -1543,20 +1605,23 @@
       <c r="E23" s="5">
         <v>43438</v>
       </c>
-      <c r="H23" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="I23" s="11"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H23" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="I23" s="10">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
       <c r="A24" s="3" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="D24" s="4">
         <v>12500</v>
@@ -1564,20 +1629,23 @@
       <c r="E24" s="5">
         <v>43441</v>
       </c>
-      <c r="H24" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="I24" s="11"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H24" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="I24" s="10">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
       <c r="A25" s="3" t="s">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="D25" s="4">
         <v>16000</v>
@@ -1586,15 +1654,15 @@
         <v>43470</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11">
       <c r="A26" s="3" t="s">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D26" s="4">
         <v>1200</v>
@@ -1603,15 +1671,15 @@
         <v>43487</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11">
       <c r="A27" s="3" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="D27" s="4">
         <v>16000</v>
@@ -1620,15 +1688,15 @@
         <v>43527</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11">
       <c r="A28" s="3" t="s">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D28" s="4">
         <v>3200</v>
@@ -1637,15 +1705,15 @@
         <v>43547</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11">
       <c r="A29" s="3" t="s">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="D29" s="4">
         <v>3200</v>
@@ -1654,15 +1722,15 @@
         <v>43552</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11">
       <c r="A30" s="3" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D30" s="4">
         <v>12500</v>
@@ -1671,15 +1739,15 @@
         <v>43557</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11">
       <c r="A31" s="3" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="D31" s="4">
         <v>12500</v>
@@ -1688,15 +1756,15 @@
         <v>43624</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11">
       <c r="A32" s="3" t="s">
-        <v>7</v>
+        <v>76</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D32" s="4">
         <v>16000</v>
@@ -1705,15 +1773,15 @@
         <v>43654</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5">
       <c r="A33" s="3" t="s">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="D33" s="4">
         <v>16000</v>
@@ -1722,15 +1790,15 @@
         <v>43655</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5">
       <c r="A34" s="3" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="D34" s="4">
         <v>12500</v>
@@ -1739,15 +1807,15 @@
         <v>43701</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5">
       <c r="A35" s="3" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D35" s="4">
         <v>1200</v>
@@ -1756,15 +1824,15 @@
         <v>43727</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5">
       <c r="A36" s="3" t="s">
-        <v>51</v>
+        <v>80</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D36" s="4">
         <v>16000</v>
@@ -1773,15 +1841,15 @@
         <v>43748</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5">
       <c r="A37" s="3" t="s">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="D37" s="4">
         <v>3200</v>
@@ -1790,15 +1858,15 @@
         <v>43758</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5">
       <c r="A38" s="3" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="D38" s="4">
         <v>12500</v>
@@ -1807,15 +1875,15 @@
         <v>43832</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5">
       <c r="A39" s="3" t="s">
-        <v>22</v>
+        <v>83</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="D39" s="4">
         <v>1200</v>
@@ -1824,15 +1892,15 @@
         <v>43877</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5">
       <c r="A40" s="3" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D40" s="4">
         <v>16000</v>
@@ -1841,15 +1909,15 @@
         <v>43880</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5">
       <c r="A41" s="3" t="s">
-        <v>38</v>
+        <v>85</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D41" s="4">
         <v>16000</v>
@@ -1858,15 +1926,15 @@
         <v>43912</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5">
       <c r="A42" s="3" t="s">
-        <v>16</v>
+        <v>86</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D42" s="4">
         <v>4600</v>
@@ -1875,15 +1943,15 @@
         <v>44020</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5">
       <c r="A43" s="3" t="s">
-        <v>41</v>
+        <v>87</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D43" s="4">
         <v>12500</v>
@@ -1892,15 +1960,15 @@
         <v>44020</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5">
       <c r="A44" s="3" t="s">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D44" s="4">
         <v>3200</v>
@@ -1909,15 +1977,15 @@
         <v>44021</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5">
       <c r="A45" s="3" t="s">
-        <v>13</v>
+        <v>89</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D45" s="4">
         <v>4600</v>
@@ -1926,15 +1994,15 @@
         <v>44089</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5">
       <c r="A46" s="3" t="s">
-        <v>46</v>
+        <v>90</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="D46" s="4">
         <v>16000</v>
@@ -1943,15 +2011,15 @@
         <v>44099</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5">
       <c r="A47" s="3" t="s">
-        <v>23</v>
+        <v>91</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D47" s="4">
         <v>12500</v>
@@ -1960,15 +2028,15 @@
         <v>44105</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5">
       <c r="A48" s="3" t="s">
-        <v>25</v>
+        <v>92</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="D48" s="4">
         <v>12500</v>
@@ -1977,15 +2045,15 @@
         <v>44128</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5">
       <c r="A49" s="3" t="s">
-        <v>21</v>
+        <v>93</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D49" s="4">
         <v>12500</v>
@@ -1994,15 +2062,15 @@
         <v>44155</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5">
       <c r="A50" s="3" t="s">
-        <v>15</v>
+        <v>94</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="D50" s="4">
         <v>12500</v>

</xml_diff>